<commit_message>
Added more data to excel and removed unwanted lines
</commit_message>
<xml_diff>
--- a/Database/Automation_856_Workflow_Data.xlsx
+++ b/Database/Automation_856_Workflow_Data.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
   <si>
     <t>OrderID</t>
   </si>
@@ -163,6 +163,15 @@
   </si>
   <si>
     <t>DC05</t>
+  </si>
+  <si>
+    <t>ORD007</t>
+  </si>
+  <si>
+    <t>ORD008</t>
+  </si>
+  <si>
+    <t>ORD009</t>
   </si>
 </sst>
 </file>
@@ -173,7 +182,7 @@
     <numFmt numFmtId="177" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="178" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,6 +199,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -251,7 +266,7 @@
       <alignment/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment/>
     </xf>
@@ -273,16 +288,20 @@
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
       <protection/>
     </xf>
   </cellXfs>
@@ -659,8 +678,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultColWidth="9.42428571428571" defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="16.2857142857143" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15">
       <c r="A1" s="1" t="s">
@@ -754,17 +776,61 @@
         <v>45305</v>
       </c>
     </row>
-    <row r="8" spans="4:4" ht="15">
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="4:4" ht="15">
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="4:4" ht="15">
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="4:4" ht="15">
-      <c r="D11" s="6"/>
+    <row r="8" spans="1:4" ht="15" customHeight="1">
+      <c r="A8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8">
+        <v>560</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="9">
+        <v>45305</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="15" customHeight="1">
+      <c r="A9" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="8">
+        <v>560</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="9">
+        <v>45305</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15" customHeight="1">
+      <c r="A10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="8">
+        <v>560</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="9">
+        <v>45305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="15" customHeight="1">
+      <c r="A11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="8">
+        <v>560</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="9">
+        <v>45305</v>
+      </c>
     </row>
     <row r="12" spans="4:4" ht="15">
       <c r="D12" s="6"/>
@@ -885,6 +951,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="9.42428571428571" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15">
       <c r="A1" s="1" t="s">
@@ -928,6 +997,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="9.42428571428571" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.5714285714286" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15">
       <c r="A1" s="1" t="s">

</xml_diff>